<commit_message>
Updation of TO-DO List
</commit_message>
<xml_diff>
--- a/todo_list.xlsx
+++ b/todo_list.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/avisek/Git_Repositary/DecodeLabs-Internship/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{822BEA0D-11BE-A341-B9BC-8B540AB2CCC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ECC78D6-400F-974A-8AA5-E87594537715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="23">
   <si>
     <t>Task ID</t>
   </si>
@@ -96,17 +96,29 @@
 statistics, analytical thinking</t>
   </si>
   <si>
-    <t>In Progress</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Missing Values replaced by No Coupon
-No Duplicates found
-Data formats okay
-outliers detected &amp; Cap outliers for premium customer identification
-Histogram for data distribution
-Correlation
-Used Python for data cleaning
-</t>
+    <t>DCLB-P2</t>
+  </si>
+  <si>
+    <t>DCLB-P3</t>
+  </si>
+  <si>
+    <t>Project 3</t>
+  </si>
+  <si>
+    <t>DA003</t>
+  </si>
+  <si>
+    <t>Goal:
+Use SQL queries to extract
+insights from a dataset.
+Key Requirements:
+• Write SELECT queries
+• Use WHERE, ORDER BY, GROUP BY
+• Perform basic aggregations
+(COUNT, SUM, AVG)
+Key Skills:
+SQL fundamentals, querying
+data, filtering and grouping</t>
   </si>
 </sst>
 </file>
@@ -470,7 +482,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.1640625" style="1" bestFit="1" customWidth="1"/>
@@ -551,13 +563,11 @@
       <c r="G3" s="2">
         <v>46109</v>
       </c>
-      <c r="H3" s="3" t="s">
-        <v>19</v>
-      </c>
+      <c r="H3" s="3"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>15</v>
@@ -589,13 +599,59 @@
         <v>8</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="E5" s="2">
         <v>46106</v>
       </c>
       <c r="G5" s="2">
         <v>46112</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="2">
+        <v>46109</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46109</v>
+      </c>
+      <c r="G6" s="2">
+        <v>46109</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="221" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="2">
+        <v>46109</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46116</v>
+      </c>
+      <c r="G7" s="2">
+        <v>46116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>